<commit_message>
works with multiple files
</commit_message>
<xml_diff>
--- a/Data_table_organiser_program/csv_file_organiser.xlsx
+++ b/Data_table_organiser_program/csv_file_organiser.xlsx
@@ -413,96 +413,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>boing</t>
+          <t>wooo</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> boing</t>
+          <t xml:space="preserve"> data</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> boing.1</t>
+          <t xml:space="preserve"> look</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> boing.2</t>
+          <t xml:space="preserve"> cool</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ouch</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Unnamed: 5</t>
+          <t>Unnamed: 4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>goober</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> bloob</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> gloop</t>
-        </is>
-      </c>
+          <t>line two</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>john</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> john</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> john</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> marcus</t>
-        </is>
-      </c>
+          <t>numbers:</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>845536746853.3749</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fweeeeeeeee</t>
+          <t>drewvogryp</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>